<commit_message>
Feature/fix participant status (#133)
Fix status check for appointment PS indiv
Add example for appointment SOS a46457b4e13a65d7f84f0ed230b6393f2ca4f870
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-FrAppointmentSAS.xlsx
+++ b/main/ig/StructureDefinition-FrAppointmentSAS.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3140" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3139" uniqueCount="473">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-15T12:59:24+00:00</t>
+    <t>2026-06-15T13:14:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1475,13 +1475,7 @@
     <t>Participation status of the actor.</t>
   </si>
   <si>
-    <t>accepted</t>
-  </si>
-  <si>
-    <t>The Participation status of an appointment.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/participationstatus|4.0.1</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/sas/ValueSet/sas-valueset-participant-status</t>
   </si>
   <si>
     <t>Appointment.participant.period</t>
@@ -1846,7 +1840,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="84.33984375" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="48.55859375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="64.7578125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
@@ -11494,7 +11488,7 @@
         <v>72</v>
       </c>
       <c r="S95" t="s" s="2">
-        <v>465</v>
+        <v>72</v>
       </c>
       <c r="T95" t="s" s="2">
         <v>72</v>
@@ -11511,11 +11505,9 @@
       <c r="X95" t="s" s="2">
         <v>205</v>
       </c>
-      <c r="Y95" t="s" s="2">
-        <v>466</v>
-      </c>
+      <c r="Y95" s="2"/>
       <c r="Z95" t="s" s="2">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="AA95" t="s" s="2">
         <v>72</v>
@@ -11550,10 +11542,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -11579,10 +11571,10 @@
         <v>294</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="N96" t="s" s="2">
         <v>297</v>
@@ -11635,7 +11627,7 @@
         <v>72</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>73</v>
@@ -11652,10 +11644,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -11681,13 +11673,13 @@
         <v>294</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="M97" t="s" s="2">
+        <v>471</v>
+      </c>
+      <c r="N97" t="s" s="2">
         <v>472</v>
-      </c>
-      <c r="M97" t="s" s="2">
-        <v>473</v>
-      </c>
-      <c r="N97" t="s" s="2">
-        <v>474</v>
       </c>
       <c r="O97" s="2"/>
       <c r="P97" t="s" s="2">
@@ -11737,7 +11729,7 @@
         <v>72</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>73</v>

</xml_diff>